<commit_message>
updated note to commissioning excel -> NTC duty to Temperature does not match Wolfspeed docs
</commit_message>
<xml_diff>
--- a/Altium/Project Outputs for uz_per_wolfspeed_25kw_FM3/Rev04/uz_per_wolfspeed_25kw_FM3_Rev04_Inbetriebnahme.xlsx
+++ b/Altium/Project Outputs for uz_per_wolfspeed_25kw_FM3/Rev04/uz_per_wolfspeed_25kw_FM3_Rev04_Inbetriebnahme.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micha\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\UltraZohm\pcb_design\uz_per_wolfspeed_25kw_fm3\Altium\Project Outputs for uz_per_wolfspeed_25kw_FM3\Rev04\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E50BE8D-244B-4566-A14A-D2EA78FCF725}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4F78D66-4B4A-48FB-9548-CF191C80A6EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28695" yWindow="-5295" windowWidth="26010" windowHeight="20985" xr2:uid="{5DF6BF0F-576E-4235-A3F4-3A36D2D7780D}"/>
+    <workbookView xWindow="32790" yWindow="-1305" windowWidth="21930" windowHeight="15225" activeTab="1" xr2:uid="{5DF6BF0F-576E-4235-A3F4-3A36D2D7780D}"/>
   </bookViews>
   <sheets>
     <sheet name="Signale" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="57">
   <si>
     <t>Inbetriebnahme Wolfspeed Interface PCB Rev04</t>
   </si>
@@ -209,13 +209,16 @@
   </si>
   <si>
     <t>A/V</t>
+  </si>
+  <si>
+    <t>5,7% dutycyc sind ca. Raumtemperatur am Wolfspeed Inverter 2.0 gemessen. Funktion oben passt also nicht !!!</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -241,6 +244,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -299,7 +310,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -308,9 +319,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -320,6 +328,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -4090,13 +4102,13 @@
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="E2" s="1" t="s">
@@ -4567,10 +4579,10 @@
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A21" s="11" t="s">
+      <c r="A21" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="B21" s="11"/>
+      <c r="B21" s="10"/>
     </row>
     <row r="22" spans="1:9" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="7" t="s">
@@ -4588,10 +4600,10 @@
         <v>37</v>
       </c>
       <c r="G22" s="7"/>
-      <c r="H22" s="9" t="s">
+      <c r="H22" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="I22" s="9"/>
+      <c r="I22" s="8"/>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" s="7" t="s">
@@ -4614,8 +4626,8 @@
         <v>36</v>
       </c>
       <c r="G23" s="7"/>
-      <c r="H23" s="9"/>
-      <c r="I23" s="9"/>
+      <c r="H23" s="8"/>
+      <c r="I23" s="8"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" s="5" t="s">
@@ -4666,7 +4678,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C4CD7F7-6135-40E0-9432-DBBFCC09CE99}">
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="32.453125" bestFit="1" customWidth="1"/>
@@ -4783,7 +4795,7 @@
         <f t="shared" si="0"/>
         <v>7.9665933440000174</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="11" t="s">
         <v>28</v>
       </c>
       <c r="E10">
@@ -4807,7 +4819,7 @@
         <f t="shared" si="0"/>
         <v>19.713728074228726</v>
       </c>
-      <c r="D11" s="8"/>
+      <c r="D11" s="11"/>
       <c r="E11">
         <f t="shared" si="2"/>
         <v>28.537085000000019</v>
@@ -4829,7 +4841,7 @@
         <f t="shared" si="0"/>
         <v>30.247141835797009</v>
       </c>
-      <c r="D12" s="8"/>
+      <c r="D12" s="11"/>
       <c r="E12">
         <f t="shared" si="2"/>
         <v>34.327574999999996</v>
@@ -4851,7 +4863,7 @@
         <f t="shared" si="0"/>
         <v>39.838175822850104</v>
       </c>
-      <c r="D13" s="8"/>
+      <c r="D13" s="11"/>
       <c r="E13">
         <f t="shared" si="2"/>
         <v>40.118065000000001</v>
@@ -4873,7 +4885,7 @@
         <f t="shared" si="0"/>
         <v>48.723912073134187</v>
       </c>
-      <c r="D14" s="8"/>
+      <c r="D14" s="11"/>
       <c r="E14">
         <f t="shared" si="2"/>
         <v>46.020629000000014</v>
@@ -4895,7 +4907,7 @@
         <f t="shared" si="0"/>
         <v>56.693108764690294</v>
       </c>
-      <c r="D15" s="8"/>
+      <c r="D15" s="11"/>
       <c r="E15">
         <f t="shared" si="2"/>
         <v>51.848477000000003</v>
@@ -4917,7 +4929,7 @@
         <f t="shared" si="0"/>
         <v>63.71950633593994</v>
       </c>
-      <c r="D16" s="8"/>
+      <c r="D16" s="11"/>
       <c r="E16">
         <f t="shared" si="2"/>
         <v>57.489535000000018</v>
@@ -4939,7 +4951,7 @@
         <f t="shared" si="0"/>
         <v>70.32381824858939</v>
       </c>
-      <c r="D17" s="8"/>
+      <c r="D17" s="11"/>
       <c r="E17">
         <f t="shared" si="2"/>
         <v>63.298704000000015</v>
@@ -4961,7 +4973,7 @@
         <f t="shared" si="0"/>
         <v>75.38978188593768</v>
       </c>
-      <c r="D18" s="8"/>
+      <c r="D18" s="11"/>
       <c r="E18">
         <f t="shared" si="2"/>
         <v>68.13656499999999</v>
@@ -4983,7 +4995,7 @@
         <f t="shared" si="0"/>
         <v>81.139753228494357</v>
       </c>
-      <c r="D19" s="8"/>
+      <c r="D19" s="11"/>
       <c r="E19">
         <f t="shared" si="2"/>
         <v>74.076487000000014</v>
@@ -5005,7 +5017,7 @@
         <f t="shared" si="0"/>
         <v>86.432776369961033</v>
       </c>
-      <c r="D20" s="8"/>
+      <c r="D20" s="11"/>
       <c r="E20">
         <f t="shared" si="2"/>
         <v>79.997730000000018</v>
@@ -5027,7 +5039,7 @@
         <f t="shared" si="0"/>
         <v>91.293730213473467</v>
       </c>
-      <c r="D21" s="8"/>
+      <c r="D21" s="11"/>
       <c r="E21">
         <f t="shared" si="2"/>
         <v>85.825578000000007</v>
@@ -5049,7 +5061,7 @@
         <f t="shared" si="0"/>
         <v>95.786341846958877</v>
       </c>
-      <c r="D22" s="8"/>
+      <c r="D22" s="11"/>
       <c r="E22">
         <f t="shared" si="2"/>
         <v>91.522672999999998</v>
@@ -5071,7 +5083,7 @@
         <f t="shared" si="0"/>
         <v>100.12360315783805</v>
       </c>
-      <c r="D23" s="8"/>
+      <c r="D23" s="11"/>
       <c r="E23">
         <f t="shared" si="2"/>
         <v>97.257126</v>
@@ -5093,7 +5105,7 @@
         <f t="shared" si="0"/>
         <v>104.41766019484243</v>
       </c>
-      <c r="D24" s="8"/>
+      <c r="D24" s="11"/>
       <c r="E24">
         <f t="shared" si="2"/>
         <v>103.084974</v>
@@ -5115,7 +5127,7 @@
         <f t="shared" si="0"/>
         <v>108.61961388335715</v>
       </c>
-      <c r="D25" s="8"/>
+      <c r="D25" s="11"/>
       <c r="E25">
         <f t="shared" si="2"/>
         <v>108.83810600000001</v>
@@ -5137,7 +5149,7 @@
         <f t="shared" si="0"/>
         <v>112.9015992397344</v>
       </c>
-      <c r="D26" s="8"/>
+      <c r="D26" s="11"/>
       <c r="E26">
         <f t="shared" si="2"/>
         <v>114.64727500000001</v>
@@ -5159,7 +5171,7 @@
         <f t="shared" si="0"/>
         <v>117.0405507145194</v>
       </c>
-      <c r="D27" s="8"/>
+      <c r="D27" s="11"/>
       <c r="E27">
         <f t="shared" si="2"/>
         <v>120.120222</v>
@@ -5181,7 +5193,7 @@
         <f t="shared" si="0"/>
         <v>121.81493000978287</v>
       </c>
-      <c r="D28" s="8"/>
+      <c r="D28" s="11"/>
       <c r="E28">
         <f t="shared" si="2"/>
         <v>126.172218</v>
@@ -5203,7 +5215,7 @@
         <f t="shared" si="0"/>
         <v>126.81635550170097</v>
       </c>
-      <c r="D29" s="8"/>
+      <c r="D29" s="11"/>
       <c r="E29">
         <f t="shared" si="2"/>
         <v>132.14949799999999</v>
@@ -5225,7 +5237,7 @@
         <f t="shared" si="0"/>
         <v>131.078741657607</v>
       </c>
-      <c r="D30" s="8"/>
+      <c r="D30" s="11"/>
       <c r="E30">
         <f t="shared" si="2"/>
         <v>136.93132199999999</v>
@@ -5247,7 +5259,7 @@
         <f t="shared" si="0"/>
         <v>136.54300995043792</v>
       </c>
-      <c r="D31" s="8"/>
+      <c r="D31" s="11"/>
       <c r="E31">
         <f t="shared" si="2"/>
         <v>142.647096</v>
@@ -5269,7 +5281,7 @@
         <f t="shared" si="0"/>
         <v>142.51937814516282</v>
       </c>
-      <c r="D32" s="8"/>
+      <c r="D32" s="11"/>
       <c r="E32">
         <f t="shared" si="2"/>
         <v>148.400228</v>
@@ -5291,7 +5303,7 @@
         <f t="shared" si="0"/>
         <v>148.65021136578559</v>
       </c>
-      <c r="D33" s="8"/>
+      <c r="D33" s="11"/>
       <c r="E33">
         <f t="shared" si="2"/>
         <v>153.817138</v>
@@ -5313,7 +5325,7 @@
         <f t="shared" si="0"/>
         <v>155.96160856290226</v>
       </c>
-      <c r="D34" s="8"/>
+      <c r="D34" s="11"/>
       <c r="E34">
         <f t="shared" si="2"/>
         <v>159.71970199999998</v>
@@ -5335,7 +5347,7 @@
         <f t="shared" si="0"/>
         <v>163.98281206510441</v>
       </c>
-      <c r="D35" s="8"/>
+      <c r="D35" s="11"/>
       <c r="E35">
         <f t="shared" si="2"/>
         <v>165.603587</v>
@@ -5357,7 +5369,7 @@
         <f t="shared" si="0"/>
         <v>172.52218312377755</v>
       </c>
-      <c r="D36" s="8"/>
+      <c r="D36" s="11"/>
       <c r="E36">
         <f t="shared" si="2"/>
         <v>171.30068199999999</v>
@@ -5379,7 +5391,7 @@
         <f t="shared" si="0"/>
         <v>181.92749510984655</v>
       </c>
-      <c r="D37" s="8"/>
+      <c r="D37" s="11"/>
       <c r="E37">
         <f t="shared" si="2"/>
         <v>177.01645600000001</v>
@@ -5401,7 +5413,7 @@
         <f t="shared" si="0"/>
         <v>192.31597887182778</v>
       </c>
-      <c r="D38" s="8"/>
+      <c r="D38" s="11"/>
       <c r="E38">
         <f t="shared" si="2"/>
         <v>182.769588</v>
@@ -5492,6 +5504,11 @@
     <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="C46" s="5" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A54" s="12" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated Inbetriebnahme sheet with assumed Temperature to PWM dutycycle function
</commit_message>
<xml_diff>
--- a/Altium/Project Outputs for uz_per_wolfspeed_25kw_FM3/Rev04/uz_per_wolfspeed_25kw_FM3_Rev04_Inbetriebnahme.xlsx
+++ b/Altium/Project Outputs for uz_per_wolfspeed_25kw_FM3/Rev04/uz_per_wolfspeed_25kw_FM3_Rev04_Inbetriebnahme.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\UltraZohm\pcb_design\uz_per_wolfspeed_25kw_fm3\Altium\Project Outputs for uz_per_wolfspeed_25kw_FM3\Rev04\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4F78D66-4B4A-48FB-9548-CF191C80A6EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B728605-747A-427E-AB5C-E7E2923B9CD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32790" yWindow="-1305" windowWidth="21930" windowHeight="15225" activeTab="1" xr2:uid="{5DF6BF0F-576E-4235-A3F4-3A36D2D7780D}"/>
+    <workbookView xWindow="22932" yWindow="-4320" windowWidth="30936" windowHeight="16776" activeTab="1" xr2:uid="{5DF6BF0F-576E-4235-A3F4-3A36D2D7780D}"/>
   </bookViews>
   <sheets>
     <sheet name="Signale" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="61">
   <si>
     <t>Inbetriebnahme Wolfspeed Interface PCB Rev04</t>
   </si>
@@ -213,6 +213,18 @@
   <si>
     <t>5,7% dutycyc sind ca. Raumtemperatur am Wolfspeed Inverter 2.0 gemessen. Funktion oben passt also nicht !!!</t>
   </si>
+  <si>
+    <t>ChatGPT estimate</t>
+  </si>
+  <si>
+    <t>duty cycle in %</t>
+  </si>
+  <si>
+    <t>T in °C</t>
+  </si>
+  <si>
+    <t>linear</t>
+  </si>
 </sst>
 </file>
 
@@ -319,6 +331,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -328,10 +344,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1949,6 +1961,585 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="de-DE"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>NTC!$B$60</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>T in °C</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-0.42941097987751531"/>
+                  <c:y val="-4.1650262467191619E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="de-DE"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>NTC!$A$61:$A$69</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>5.7</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>8.8000000000000007</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>15.7</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>23.4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>31.5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>43.6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>60.8</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>72.900000000000006</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>80.7</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>NTC!$B$61:$B$69</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>24.999074838492277</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>30.048089614535002</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>40.018523362193662</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>49.9970424077502</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>59.958388211798479</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>74.990552568002443</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>99.937177386569203</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>124.80658015741955</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>149.78982168995555</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-B2EC-45CA-BB53-B8D729E27BEC}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>T in °C lin.</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>NTC!$A$61:$A$69</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>5.7</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>8.8000000000000007</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>15.7</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>23.4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>31.5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>43.6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>60.8</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>72.900000000000006</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>80.7</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>NTC!$C$61:$C$69</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>22.474</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>27.279000000000003</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>37.974000000000004</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>49.908999999999992</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>62.463999999999999</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>81.218999999999994</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>107.87899999999999</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>126.63400000000001</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>138.72400000000002</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-B2EC-45CA-BB53-B8D729E27BEC}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1267785535"/>
+        <c:axId val="1267779775"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1267785535"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="de-DE"/>
+                  <a:t>duty cycle in %</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="de-DE"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="de-DE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1267779775"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1267779775"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="de-DE"/>
+                  <a:t>Temperature in °C</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="de-DE"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="de-DE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1267785535"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="de-DE"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.78740157499999996" l="0.7" r="0.7" t="0.78740157499999996" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -2069,6 +2660,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -3102,6 +3733,522 @@
 </file>
 
 <file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -3700,9 +4847,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>447969</xdr:colOff>
+      <xdr:colOff>441619</xdr:colOff>
       <xdr:row>48</xdr:row>
-      <xdr:rowOff>123846</xdr:rowOff>
+      <xdr:rowOff>137816</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3766,6 +4913,174 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>91440</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>200660</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>383868</xdr:colOff>
+      <xdr:row>85</xdr:row>
+      <xdr:rowOff>21887</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Grafik 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{322988BA-5E68-24C1-4FFB-6A725FE987CB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10744200" y="9893300"/>
+          <a:ext cx="6388428" cy="5795307"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>116840</xdr:colOff>
+      <xdr:row>84</xdr:row>
+      <xdr:rowOff>138430</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>459993</xdr:colOff>
+      <xdr:row>112</xdr:row>
+      <xdr:rowOff>20577</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Grafik 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5368DE6D-49D1-1884-21C4-98D78985AA40}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10769600" y="15614650"/>
+          <a:ext cx="4915153" cy="4998977"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>434340</xdr:colOff>
+      <xdr:row>78</xdr:row>
+      <xdr:rowOff>161290</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>251762</xdr:colOff>
+      <xdr:row>89</xdr:row>
+      <xdr:rowOff>135991</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Grafik 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8DD61902-C11B-8936-73B7-E3026DF3C256}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="434340" y="14540230"/>
+          <a:ext cx="5885482" cy="1972411"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>462280</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>58420</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>462280</xdr:colOff>
+      <xdr:row>73</xdr:row>
+      <xdr:rowOff>58420</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="9" name="Diagramm 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{96DF479C-F821-E658-38D6-5F641F7A7496}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -4102,13 +5417,13 @@
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="E2" s="1" t="s">
@@ -4579,10 +5894,10 @@
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A21" s="10" t="s">
+      <c r="A21" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="B21" s="10"/>
+      <c r="B21" s="12"/>
     </row>
     <row r="22" spans="1:9" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="7" t="s">
@@ -4600,10 +5915,10 @@
         <v>37</v>
       </c>
       <c r="G22" s="7"/>
-      <c r="H22" s="8" t="s">
+      <c r="H22" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="I22" s="8"/>
+      <c r="I22" s="10"/>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" s="7" t="s">
@@ -4626,8 +5941,8 @@
         <v>36</v>
       </c>
       <c r="G23" s="7"/>
-      <c r="H23" s="8"/>
-      <c r="I23" s="8"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="10"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" s="5" t="s">
@@ -4678,7 +5993,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C4CD7F7-6135-40E0-9432-DBBFCC09CE99}">
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="32.453125" bestFit="1" customWidth="1"/>
@@ -4795,7 +6110,7 @@
         <f t="shared" si="0"/>
         <v>7.9665933440000174</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="9" t="s">
         <v>28</v>
       </c>
       <c r="E10">
@@ -4819,7 +6134,7 @@
         <f t="shared" si="0"/>
         <v>19.713728074228726</v>
       </c>
-      <c r="D11" s="11"/>
+      <c r="D11" s="9"/>
       <c r="E11">
         <f t="shared" si="2"/>
         <v>28.537085000000019</v>
@@ -4841,7 +6156,7 @@
         <f t="shared" si="0"/>
         <v>30.247141835797009</v>
       </c>
-      <c r="D12" s="11"/>
+      <c r="D12" s="9"/>
       <c r="E12">
         <f t="shared" si="2"/>
         <v>34.327574999999996</v>
@@ -4863,7 +6178,7 @@
         <f t="shared" si="0"/>
         <v>39.838175822850104</v>
       </c>
-      <c r="D13" s="11"/>
+      <c r="D13" s="9"/>
       <c r="E13">
         <f t="shared" si="2"/>
         <v>40.118065000000001</v>
@@ -4885,7 +6200,7 @@
         <f t="shared" si="0"/>
         <v>48.723912073134187</v>
       </c>
-      <c r="D14" s="11"/>
+      <c r="D14" s="9"/>
       <c r="E14">
         <f t="shared" si="2"/>
         <v>46.020629000000014</v>
@@ -4907,7 +6222,7 @@
         <f t="shared" si="0"/>
         <v>56.693108764690294</v>
       </c>
-      <c r="D15" s="11"/>
+      <c r="D15" s="9"/>
       <c r="E15">
         <f t="shared" si="2"/>
         <v>51.848477000000003</v>
@@ -4929,7 +6244,7 @@
         <f t="shared" si="0"/>
         <v>63.71950633593994</v>
       </c>
-      <c r="D16" s="11"/>
+      <c r="D16" s="9"/>
       <c r="E16">
         <f t="shared" si="2"/>
         <v>57.489535000000018</v>
@@ -4951,7 +6266,7 @@
         <f t="shared" si="0"/>
         <v>70.32381824858939</v>
       </c>
-      <c r="D17" s="11"/>
+      <c r="D17" s="9"/>
       <c r="E17">
         <f t="shared" si="2"/>
         <v>63.298704000000015</v>
@@ -4973,7 +6288,7 @@
         <f t="shared" si="0"/>
         <v>75.38978188593768</v>
       </c>
-      <c r="D18" s="11"/>
+      <c r="D18" s="9"/>
       <c r="E18">
         <f t="shared" si="2"/>
         <v>68.13656499999999</v>
@@ -4995,7 +6310,7 @@
         <f t="shared" si="0"/>
         <v>81.139753228494357</v>
       </c>
-      <c r="D19" s="11"/>
+      <c r="D19" s="9"/>
       <c r="E19">
         <f t="shared" si="2"/>
         <v>74.076487000000014</v>
@@ -5017,7 +6332,7 @@
         <f t="shared" si="0"/>
         <v>86.432776369961033</v>
       </c>
-      <c r="D20" s="11"/>
+      <c r="D20" s="9"/>
       <c r="E20">
         <f t="shared" si="2"/>
         <v>79.997730000000018</v>
@@ -5039,7 +6354,7 @@
         <f t="shared" si="0"/>
         <v>91.293730213473467</v>
       </c>
-      <c r="D21" s="11"/>
+      <c r="D21" s="9"/>
       <c r="E21">
         <f t="shared" si="2"/>
         <v>85.825578000000007</v>
@@ -5061,7 +6376,7 @@
         <f t="shared" si="0"/>
         <v>95.786341846958877</v>
       </c>
-      <c r="D22" s="11"/>
+      <c r="D22" s="9"/>
       <c r="E22">
         <f t="shared" si="2"/>
         <v>91.522672999999998</v>
@@ -5083,7 +6398,7 @@
         <f t="shared" si="0"/>
         <v>100.12360315783805</v>
       </c>
-      <c r="D23" s="11"/>
+      <c r="D23" s="9"/>
       <c r="E23">
         <f t="shared" si="2"/>
         <v>97.257126</v>
@@ -5105,7 +6420,7 @@
         <f t="shared" si="0"/>
         <v>104.41766019484243</v>
       </c>
-      <c r="D24" s="11"/>
+      <c r="D24" s="9"/>
       <c r="E24">
         <f t="shared" si="2"/>
         <v>103.084974</v>
@@ -5127,7 +6442,7 @@
         <f t="shared" si="0"/>
         <v>108.61961388335715</v>
       </c>
-      <c r="D25" s="11"/>
+      <c r="D25" s="9"/>
       <c r="E25">
         <f t="shared" si="2"/>
         <v>108.83810600000001</v>
@@ -5149,7 +6464,7 @@
         <f t="shared" si="0"/>
         <v>112.9015992397344</v>
       </c>
-      <c r="D26" s="11"/>
+      <c r="D26" s="9"/>
       <c r="E26">
         <f t="shared" si="2"/>
         <v>114.64727500000001</v>
@@ -5171,7 +6486,7 @@
         <f t="shared" si="0"/>
         <v>117.0405507145194</v>
       </c>
-      <c r="D27" s="11"/>
+      <c r="D27" s="9"/>
       <c r="E27">
         <f t="shared" si="2"/>
         <v>120.120222</v>
@@ -5193,7 +6508,7 @@
         <f t="shared" si="0"/>
         <v>121.81493000978287</v>
       </c>
-      <c r="D28" s="11"/>
+      <c r="D28" s="9"/>
       <c r="E28">
         <f t="shared" si="2"/>
         <v>126.172218</v>
@@ -5215,7 +6530,7 @@
         <f t="shared" si="0"/>
         <v>126.81635550170097</v>
       </c>
-      <c r="D29" s="11"/>
+      <c r="D29" s="9"/>
       <c r="E29">
         <f t="shared" si="2"/>
         <v>132.14949799999999</v>
@@ -5237,7 +6552,7 @@
         <f t="shared" si="0"/>
         <v>131.078741657607</v>
       </c>
-      <c r="D30" s="11"/>
+      <c r="D30" s="9"/>
       <c r="E30">
         <f t="shared" si="2"/>
         <v>136.93132199999999</v>
@@ -5259,7 +6574,7 @@
         <f t="shared" si="0"/>
         <v>136.54300995043792</v>
       </c>
-      <c r="D31" s="11"/>
+      <c r="D31" s="9"/>
       <c r="E31">
         <f t="shared" si="2"/>
         <v>142.647096</v>
@@ -5281,7 +6596,7 @@
         <f t="shared" si="0"/>
         <v>142.51937814516282</v>
       </c>
-      <c r="D32" s="11"/>
+      <c r="D32" s="9"/>
       <c r="E32">
         <f t="shared" si="2"/>
         <v>148.400228</v>
@@ -5303,7 +6618,7 @@
         <f t="shared" si="0"/>
         <v>148.65021136578559</v>
       </c>
-      <c r="D33" s="11"/>
+      <c r="D33" s="9"/>
       <c r="E33">
         <f t="shared" si="2"/>
         <v>153.817138</v>
@@ -5325,7 +6640,7 @@
         <f t="shared" si="0"/>
         <v>155.96160856290226</v>
       </c>
-      <c r="D34" s="11"/>
+      <c r="D34" s="9"/>
       <c r="E34">
         <f t="shared" si="2"/>
         <v>159.71970199999998</v>
@@ -5347,7 +6662,7 @@
         <f t="shared" si="0"/>
         <v>163.98281206510441</v>
       </c>
-      <c r="D35" s="11"/>
+      <c r="D35" s="9"/>
       <c r="E35">
         <f t="shared" si="2"/>
         <v>165.603587</v>
@@ -5369,7 +6684,7 @@
         <f t="shared" si="0"/>
         <v>172.52218312377755</v>
       </c>
-      <c r="D36" s="11"/>
+      <c r="D36" s="9"/>
       <c r="E36">
         <f t="shared" si="2"/>
         <v>171.30068199999999</v>
@@ -5391,7 +6706,7 @@
         <f t="shared" si="0"/>
         <v>181.92749510984655</v>
       </c>
-      <c r="D37" s="11"/>
+      <c r="D37" s="9"/>
       <c r="E37">
         <f t="shared" si="2"/>
         <v>177.01645600000001</v>
@@ -5413,7 +6728,7 @@
         <f t="shared" si="0"/>
         <v>192.31597887182778</v>
       </c>
-      <c r="D38" s="11"/>
+      <c r="D38" s="9"/>
       <c r="E38">
         <f t="shared" si="2"/>
         <v>182.769588</v>
@@ -5506,9 +6821,142 @@
         <v>29</v>
       </c>
     </row>
-    <row r="54" spans="1:1" ht="23.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A54" s="12" t="s">
+    <row r="54" spans="1:3" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A54" s="8" t="s">
         <v>56</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
+        <v>58</v>
+      </c>
+      <c r="B60" t="s">
+        <v>59</v>
+      </c>
+      <c r="C60" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A61">
+        <v>5.7</v>
+      </c>
+      <c r="B61">
+        <f>1/(1/298.15+1/3525*LN((7912171.1-83286*A61)/(5000*(84.1273*A61+1007.908))))-273.15</f>
+        <v>24.999074838492277</v>
+      </c>
+      <c r="C61">
+        <f>1.55*A61+13.639</f>
+        <v>22.474</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A62">
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="B62">
+        <f t="shared" ref="B62:B79" si="4">1/(1/298.15+1/3525*LN((7912171.1-83286*A62)/(5000*(84.1273*A62+1007.908))))-273.15</f>
+        <v>30.048089614535002</v>
+      </c>
+      <c r="C62">
+        <f t="shared" ref="C62:C69" si="5">1.55*A62+13.639</f>
+        <v>27.279000000000003</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A63">
+        <v>15.7</v>
+      </c>
+      <c r="B63">
+        <f t="shared" si="4"/>
+        <v>40.018523362193662</v>
+      </c>
+      <c r="C63">
+        <f t="shared" si="5"/>
+        <v>37.974000000000004</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A64">
+        <v>23.4</v>
+      </c>
+      <c r="B64">
+        <f t="shared" si="4"/>
+        <v>49.9970424077502</v>
+      </c>
+      <c r="C64">
+        <f t="shared" si="5"/>
+        <v>49.908999999999992</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A65">
+        <v>31.5</v>
+      </c>
+      <c r="B65">
+        <f t="shared" si="4"/>
+        <v>59.958388211798479</v>
+      </c>
+      <c r="C65">
+        <f t="shared" si="5"/>
+        <v>62.463999999999999</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A66">
+        <v>43.6</v>
+      </c>
+      <c r="B66">
+        <f t="shared" si="4"/>
+        <v>74.990552568002443</v>
+      </c>
+      <c r="C66">
+        <f t="shared" si="5"/>
+        <v>81.218999999999994</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A67">
+        <v>60.8</v>
+      </c>
+      <c r="B67">
+        <f t="shared" si="4"/>
+        <v>99.937177386569203</v>
+      </c>
+      <c r="C67">
+        <f t="shared" si="5"/>
+        <v>107.87899999999999</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A68">
+        <v>72.900000000000006</v>
+      </c>
+      <c r="B68">
+        <f t="shared" si="4"/>
+        <v>124.80658015741955</v>
+      </c>
+      <c r="C68">
+        <f t="shared" si="5"/>
+        <v>126.63400000000001</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A69">
+        <v>80.7</v>
+      </c>
+      <c r="B69">
+        <f t="shared" si="4"/>
+        <v>149.78982168995555</v>
+      </c>
+      <c r="C69">
+        <f t="shared" si="5"/>
+        <v>138.72400000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>